<commit_message>
Generalize excel_formula pipeline to 00a-09 ticker-parameterized scripts
Renames 04/05/08 from TSLA/TSLL-specific scripts to generic <TICKER>-arg
versions (05_prep_ticker_bdh_full, 08_fetch_ticker_spot_yfinance,
09_fetch_ticker_ohlcv_yfinance), splits the Excel5 template builder into
00a and adds 00b_build_excel3 to generate the Excel3 BDH formula template,
and syncs README.md with the new 00a-00b/01-03/05-09 numbering.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel_formula/Excel3_Underlying_Data.xlsx
+++ b/excel_formula/Excel3_Underlying_Data.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSTR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMCI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSLA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COIN" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLTR" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MU" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ETH" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NG1" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOXX" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AVGO" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVO" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVDA" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSOS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MSTR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SMCI" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TSLA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="COIN" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PLTR" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MU" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ETH" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="NG1" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SOXX" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AVGO" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="NVO" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="NVDA" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="MSOS" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +46,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
@@ -69,6 +68,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -84,18 +84,17 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <i val="1"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +123,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
@@ -148,10 +152,10 @@
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -159,25 +163,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1662,6 +1666,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2770,6 +2775,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2924,6 +2930,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>